<commit_message>
hito 2026-09-19 17:49 · 4 files changed 57 insertions(+) 3 deletions(-)
</commit_message>
<xml_diff>
--- a/datos_congreso.xlsx
+++ b/datos_congreso.xlsx
@@ -7620,7 +7620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7954,6 +7954,36 @@
       </c>
       <c r="C32" t="n">
         <v>10</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>16857-07</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Modifica el Código Penal para autorizar el uso de agentes encubiertos en Internet para la persecución de delitos sexuales contra niños, niñas y adolescentes</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>18137-05</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Adopta medidas transitorias para contener el precio del kerosene doméstico en el contexto de la emergencia energética internacional, y otras medidas que indica</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>